<commit_message>
Updated IND_grids_syn_5 model - 2025-11-07 13:54
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_syn_5/Sets-vervestacks.xlsx
+++ b/VerveStacks_IND_grids_syn_5/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_syn_5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C43C13E-E72B-46CA-97BE-F81F75295404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CBD5898F-CF77-4955-A23D-635BA37D6919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3275,7 +3275,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E6B9-8DFD-4214-A3CC-5D5D6B730333}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A1DB11D-2E61-4186-9420-C6E2BA6910E2}">
   <dimension ref="B9:E358"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>